<commit_message>
test: normalize english checklist fixtures
</commit_message>
<xml_diff>
--- a/tests/fixtures/import/review_checklist_import/english-excel.xlsx
+++ b/tests/fixtures/import/review_checklist_import/english-excel.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审查清单" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="补充说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -55,16 +54,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -431,17 +427,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="78" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>清单名称</t>
@@ -456,7 +452,7 @@
       <c r="D1" s="1" t="n"/>
       <c r="E1" s="1" t="n"/>
     </row>
-    <row r="2">
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>适用合同类型</t>
@@ -464,14 +460,14 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Sales Agreement</t>
+          <t>Procurement Agreement</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
       <c r="D2" s="1" t="n"/>
       <c r="E2" s="1" t="n"/>
     </row>
-    <row r="3">
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>说明</t>
@@ -486,14 +482,14 @@
       <c r="D3" s="1" t="n"/>
       <c r="E3" s="1" t="n"/>
     </row>
-    <row r="4">
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" s="1" t="n"/>
       <c r="B4" s="1" t="n"/>
       <c r="C4" s="1" t="n"/>
       <c r="D4" s="1" t="n"/>
       <c r="E4" s="1" t="n"/>
     </row>
-    <row r="5">
+    <row r="5" ht="24" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>序号</t>
@@ -520,59 +516,128 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="24" customHeight="1">
       <c r="A6" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Confidentiality Notice Must Remain in English</t>
+          <t>Confidentiality obligation</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>The supplier shall keep all confidential information strictly protected and shall notify the buyer before any disclosure.</t>
+          <t>The agreement must include an English confidentiality clause covering confidential information, disclosure restrictions, survival period, and permitted recipients.</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>Request legal review before approval when the confidentiality clause is missing.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>补充规则</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>The checklist language must remain English after import.</t>
+          <t>Flag the contract as high risk if confidential information can be disclosed without prior written consent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Payment schedule</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Payment milestones, invoice requirements, tax treatment, currency, and late-payment consequences must be stated in clear English.</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Require finance and legal review when payment timing, amount, or invoice conditions are ambiguous.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Delivery and acceptance</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>The contract must define delivery date, delivery location, acceptance criteria, inspection period, and rejection procedure.</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Ask the business owner to add objective acceptance standards before approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Intellectual property ownership</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Ownership of deliverables, background technology, license scope, and restrictions on third-party materials must be allocated expressly.</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Escalate to legal if ownership or license rights are missing or inconsistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Termination and liability</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Termination triggers, notice period, cure period, liability cap, excluded damages, and survival obligations must be complete.</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Request revisions when termination rights or liability boundaries are one-sided or undefined.</t>
         </is>
       </c>
     </row>

</xml_diff>